<commit_message>
Fixed alias property conversion
</commit_message>
<xml_diff>
--- a/UD_CustomDevices.EspToExcel/Data/UD_DevicesEmpty.xlsx
+++ b/UD_CustomDevices.EspToExcel/Data/UD_DevicesEmpty.xlsx
@@ -20,7 +20,7 @@
     <definedName name="List_ModOutcomes">#REF!</definedName>
     <definedName name="List_ModTriggers">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <x:ext xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="87">
   <si>
     <t>EditorID</t>
   </si>
@@ -77,9 +77,6 @@
     <t>UD_DeviceAbilities_Flags</t>
   </si>
   <si>
-    <t>UD_DeviceKeyword_Minor</t>
-  </si>
-  <si>
     <t>UD_Durability_Damage_Base</t>
   </si>
   <si>
@@ -98,27 +95,6 @@
     <t>UD_MessageDeviceInteractionWH</t>
   </si>
   <si>
-    <t>UD_ModifiersDataForm1</t>
-  </si>
-  <si>
-    <t>UD_ModifiersDataForm2</t>
-  </si>
-  <si>
-    <t>UD_ModifiersDataForm3</t>
-  </si>
-  <si>
-    <t>UD_ModifiersDataForm4</t>
-  </si>
-  <si>
-    <t>UD_ModifiersDataForm5</t>
-  </si>
-  <si>
-    <t>UD_ModifiersDataStr</t>
-  </si>
-  <si>
-    <t>UD_ModifiersRef</t>
-  </si>
-  <si>
     <t>UD_ResistMagicka</t>
   </si>
   <si>
@@ -159,6 +135,162 @@
   </si>
   <si>
     <t>string[]</t>
+  </si>
+  <si>
+    <t>UD_DevcieKeyword_Minor</t>
+  </si>
+  <si>
+    <t>UD_ModifiersRef[0]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataStr[0]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm1[0]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm2[0]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm3[0]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm4[0]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm5[0]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersRef[1]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataStr[1]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm1[1]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm2[1]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm3[1]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm4[1]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm5[1]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersRef[2]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataStr[2]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm1[2]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm2[2]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm3[2]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm4[2]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm5[2]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersRef[3]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataStr[3]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm1[3]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm2[3]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm3[3]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm4[3]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm5[3]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersRef[4]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataStr[4]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm1[4]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm2[4]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm3[4]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm4[4]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm5[4]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersRef[5]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataStr[5]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm1[5]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm2[5]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm3[5]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm4[5]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm5[5]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersRef[6]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataStr[6]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm1[6]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm2[6]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm3[6]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm4[6]</t>
+  </si>
+  <si>
+    <t>UD_ModifiersDataForm5[6]</t>
+  </si>
+  <si>
+    <t>alias</t>
+  </si>
+  <si>
+    <t>string</t>
   </si>
 </sst>
 </file>
@@ -297,7 +429,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -314,18 +446,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -334,6 +454,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -596,7 +725,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:AJ6"/>
+  <dimension ref="B2:BY6"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.21875" style="1" customWidth="1"/>
@@ -607,272 +736,479 @@
     <col min="6" max="16" width="27.44140625" style="1" customWidth="1"/>
     <col min="17" max="18" width="31" style="1" customWidth="1"/>
     <col min="19" max="21" width="27.44140625" style="1" customWidth="1"/>
-    <col min="22" max="36" width="33" style="1" customWidth="1"/>
-    <col min="37" max="16384" width="8.88671875" style="1"/>
+    <col min="22" max="24" width="33" style="1" customWidth="1"/>
+    <col min="25" max="73" width="25.88671875" style="1" customWidth="1"/>
+    <col min="74" max="77" width="30.5546875" style="1" customWidth="1"/>
+    <col min="78" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:36" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="7" t="s">
+    <row r="2" spans="2:77" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="9"/>
-      <c r="D2" s="7" t="s">
+      <c r="C2" s="10"/>
+      <c r="D2" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
-      <c r="M2" s="8"/>
-      <c r="N2" s="8"/>
-      <c r="O2" s="8"/>
-      <c r="P2" s="8"/>
-      <c r="Q2" s="8"/>
-      <c r="R2" s="8"/>
-      <c r="S2" s="8"/>
-      <c r="T2" s="8"/>
-      <c r="U2" s="8"/>
-      <c r="V2" s="8"/>
-      <c r="W2" s="8"/>
-      <c r="X2" s="8"/>
-      <c r="Y2" s="8"/>
-      <c r="Z2" s="8"/>
-      <c r="AA2" s="8"/>
-      <c r="AB2" s="8"/>
-      <c r="AC2" s="8"/>
-      <c r="AD2" s="8"/>
-      <c r="AE2" s="8"/>
-      <c r="AF2" s="8"/>
-      <c r="AG2" s="8"/>
-      <c r="AH2" s="8"/>
-      <c r="AI2" s="8"/>
-      <c r="AJ2" s="9"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="11"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="11"/>
+      <c r="M2" s="11"/>
+      <c r="N2" s="11"/>
+      <c r="O2" s="11"/>
+      <c r="P2" s="11"/>
+      <c r="Q2" s="11"/>
+      <c r="R2" s="11"/>
+      <c r="S2" s="11"/>
+      <c r="T2" s="11"/>
+      <c r="U2" s="11"/>
+      <c r="V2" s="11"/>
+      <c r="W2" s="11"/>
+      <c r="X2" s="11"/>
+      <c r="Y2" s="11"/>
+      <c r="Z2" s="11"/>
+      <c r="AA2" s="11"/>
+      <c r="AB2" s="11"/>
+      <c r="AC2" s="11"/>
+      <c r="AD2" s="11"/>
+      <c r="AE2" s="11"/>
+      <c r="AF2" s="11"/>
+      <c r="AG2" s="11"/>
+      <c r="AH2" s="11"/>
+      <c r="AI2" s="11"/>
+      <c r="AJ2" s="11"/>
+      <c r="AK2" s="11"/>
+      <c r="AL2" s="11"/>
+      <c r="AM2" s="11"/>
+      <c r="AN2" s="11"/>
+      <c r="AO2" s="11"/>
+      <c r="AP2" s="11"/>
+      <c r="AQ2" s="11"/>
+      <c r="AR2" s="11"/>
+      <c r="AS2" s="11"/>
+      <c r="AT2" s="11"/>
+      <c r="AU2" s="11"/>
+      <c r="AV2" s="11"/>
+      <c r="AW2" s="11"/>
+      <c r="AX2" s="11"/>
+      <c r="AY2" s="11"/>
+      <c r="AZ2" s="11"/>
+      <c r="BA2" s="11"/>
+      <c r="BB2" s="11"/>
+      <c r="BC2" s="11"/>
+      <c r="BD2" s="11"/>
+      <c r="BE2" s="11"/>
+      <c r="BF2" s="11"/>
+      <c r="BG2" s="11"/>
+      <c r="BH2" s="11"/>
+      <c r="BI2" s="11"/>
+      <c r="BJ2" s="11"/>
+      <c r="BK2" s="11"/>
+      <c r="BL2" s="11"/>
+      <c r="BM2" s="11"/>
+      <c r="BN2" s="11"/>
+      <c r="BO2" s="11"/>
+      <c r="BP2" s="11"/>
+      <c r="BQ2" s="11"/>
+      <c r="BR2" s="11"/>
+      <c r="BS2" s="11"/>
+      <c r="BT2" s="11"/>
+      <c r="BU2" s="11"/>
+      <c r="BV2" s="11"/>
+      <c r="BW2" s="11"/>
+      <c r="BX2" s="11"/>
+      <c r="BY2" s="11"/>
     </row>
-    <row r="3" spans="2:36" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="10" t="s">
+    <row r="3" spans="2:77" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-      <c r="L3" s="8"/>
-      <c r="M3" s="8"/>
-      <c r="N3" s="8"/>
-      <c r="O3" s="8"/>
-      <c r="P3" s="8"/>
-      <c r="Q3" s="8"/>
-      <c r="R3" s="8"/>
-      <c r="S3" s="8"/>
-      <c r="T3" s="8"/>
-      <c r="U3" s="8"/>
-      <c r="V3" s="8"/>
-      <c r="W3" s="8"/>
-      <c r="X3" s="8"/>
-      <c r="Y3" s="8"/>
-      <c r="Z3" s="8"/>
-      <c r="AA3" s="8"/>
-      <c r="AB3" s="8"/>
-      <c r="AC3" s="8"/>
-      <c r="AD3" s="8"/>
-      <c r="AE3" s="8"/>
-      <c r="AF3" s="8"/>
-      <c r="AG3" s="8"/>
-      <c r="AH3" s="8"/>
-      <c r="AI3" s="8"/>
-      <c r="AJ3" s="9"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="11"/>
+      <c r="M3" s="11"/>
+      <c r="N3" s="11"/>
+      <c r="O3" s="11"/>
+      <c r="P3" s="11"/>
+      <c r="Q3" s="11"/>
+      <c r="R3" s="11"/>
+      <c r="S3" s="11"/>
+      <c r="T3" s="11"/>
+      <c r="U3" s="11"/>
+      <c r="V3" s="11"/>
+      <c r="W3" s="11"/>
+      <c r="X3" s="11"/>
+      <c r="Y3" s="11"/>
+      <c r="Z3" s="11"/>
+      <c r="AA3" s="11"/>
+      <c r="AB3" s="11"/>
+      <c r="AC3" s="11"/>
+      <c r="AD3" s="11"/>
+      <c r="AE3" s="11"/>
+      <c r="AF3" s="11"/>
+      <c r="AG3" s="11"/>
+      <c r="AH3" s="11"/>
+      <c r="AI3" s="11"/>
+      <c r="AJ3" s="11"/>
+      <c r="AK3" s="11"/>
+      <c r="AL3" s="11"/>
+      <c r="AM3" s="11"/>
+      <c r="AN3" s="11"/>
+      <c r="AO3" s="11"/>
+      <c r="AP3" s="11"/>
+      <c r="AQ3" s="11"/>
+      <c r="AR3" s="11"/>
+      <c r="AS3" s="11"/>
+      <c r="AT3" s="11"/>
+      <c r="AU3" s="11"/>
+      <c r="AV3" s="11"/>
+      <c r="AW3" s="11"/>
+      <c r="AX3" s="11"/>
+      <c r="AY3" s="11"/>
+      <c r="AZ3" s="11"/>
+      <c r="BA3" s="11"/>
+      <c r="BB3" s="11"/>
+      <c r="BC3" s="11"/>
+      <c r="BD3" s="11"/>
+      <c r="BE3" s="11"/>
+      <c r="BF3" s="11"/>
+      <c r="BG3" s="11"/>
+      <c r="BH3" s="11"/>
+      <c r="BI3" s="11"/>
+      <c r="BJ3" s="11"/>
+      <c r="BK3" s="11"/>
+      <c r="BL3" s="11"/>
+      <c r="BM3" s="11"/>
+      <c r="BN3" s="11"/>
+      <c r="BO3" s="11"/>
+      <c r="BP3" s="11"/>
+      <c r="BQ3" s="11"/>
+      <c r="BR3" s="11"/>
+      <c r="BS3" s="11"/>
+      <c r="BT3" s="11"/>
+      <c r="BU3" s="11"/>
+      <c r="BV3" s="11"/>
+      <c r="BW3" s="11"/>
+      <c r="BX3" s="11"/>
+      <c r="BY3" s="11"/>
     </row>
-    <row r="4" spans="2:36" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
+    <row r="4" spans="2:77" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
       <c r="E4" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F4" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="H4" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="I4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="J4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="K4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="K4" s="4" t="s">
+      <c r="L4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L4" s="4" t="s">
+      <c r="M4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="M4" s="4" t="s">
+      <c r="N4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="N4" s="4" t="s">
+      <c r="O4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="O4" s="4" t="s">
+      <c r="P4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="P4" s="4" t="s">
+      <c r="Q4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="R4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="S4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="T4" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="U4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="V4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="W4" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="X4" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="Y4" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z4" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA4" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB4" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="AC4" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AD4" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="AE4" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF4" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG4" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="AH4" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="AI4" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="AJ4" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK4" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="AL4" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM4" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="AN4" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="AO4" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="AP4" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ4" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="AR4" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="AS4" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT4" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="AU4" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AV4" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="AW4" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AX4" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="AY4" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="AZ4" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="BA4" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="BB4" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="BC4" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="BD4" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="BE4" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="BF4" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="BG4" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="BH4" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="BI4" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="BJ4" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="BK4" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="BL4" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="BM4" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="BN4" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="BO4" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="BP4" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="BQ4" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="BR4" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="BS4" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="BT4" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="BU4" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="BV4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="Q4" s="4" t="s">
+      <c r="BW4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="R4" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="S4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="T4" s="4" t="s">
+      <c r="BX4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="U4" s="4" t="s">
+      <c r="BY4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="V4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="W4" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="X4" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="Y4" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA4" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="AB4" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="AC4" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="AD4" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="AE4" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="AF4" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="AG4" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="AH4" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="AI4" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AJ4" s="4" t="s">
-        <v>38</v>
-      </c>
     </row>
-    <row r="5" spans="2:36" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:77" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B5" s="5"/>
-      <c r="C5" s="6"/>
+      <c r="C5" s="5"/>
       <c r="D5" s="5"/>
       <c r="E5" s="4" t="s">
         <v>4</v>
       </c>
       <c r="F5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="4" t="s">
-        <v>39</v>
-      </c>
       <c r="H5" s="4" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>5</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="M5" s="4" t="s">
         <v>5</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="O5" s="4" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="P5" s="4" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="Q5" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R5" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S5" s="4" t="s">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="T5" s="4" t="s">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="U5" s="4" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="V5" s="4" t="s">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="W5" s="4" t="s">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="X5" s="4" t="s">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="Y5" s="4" t="s">
-        <v>42</v>
+        <v>85</v>
       </c>
       <c r="Z5" s="4" t="s">
-        <v>40</v>
+        <v>86</v>
       </c>
       <c r="AA5" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AB5" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AC5" s="4" t="s">
         <v>4</v>
@@ -881,25 +1217,148 @@
         <v>4</v>
       </c>
       <c r="AE5" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AF5" s="4" t="s">
-        <v>5</v>
+        <v>85</v>
       </c>
       <c r="AG5" s="4" t="s">
-        <v>39</v>
+        <v>86</v>
       </c>
       <c r="AH5" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AI5" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AJ5" s="4" t="s">
         <v>4</v>
       </c>
+      <c r="AK5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="AL5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="AM5" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="AN5" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="AO5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="AP5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="AQ5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="AR5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="AS5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="AT5" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="AU5" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="AV5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="AW5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="AX5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="AY5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="AZ5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BA5" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="BB5" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="BC5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BD5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BE5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BF5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BG5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BH5" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="BI5" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="BJ5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BK5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BL5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BM5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BN5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BO5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BP5" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="BQ5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BR5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BS5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BT5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BU5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BV5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BW5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BX5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BY5" s="4" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="6" spans="2:36" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:77" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B6" s="4">
         <v>1</v>
       </c>
@@ -916,22 +1375,22 @@
         <v>5</v>
       </c>
       <c r="G6" s="4">
+        <v>5</v>
+      </c>
+      <c r="H6" s="4">
         <v>6</v>
       </c>
-      <c r="H6" s="4">
+      <c r="I6" s="4">
         <v>7</v>
       </c>
-      <c r="I6" s="4">
+      <c r="J6" s="4">
         <v>8</v>
       </c>
-      <c r="J6" s="4">
+      <c r="K6" s="4">
         <v>9</v>
       </c>
-      <c r="K6" s="4">
+      <c r="L6" s="4">
         <v>10</v>
-      </c>
-      <c r="L6" s="4">
-        <v>11</v>
       </c>
       <c r="M6" s="4">
         <v>12</v>
@@ -1004,6 +1463,129 @@
       </c>
       <c r="AJ6" s="4">
         <v>35</v>
+      </c>
+      <c r="AK6" s="4">
+        <v>36</v>
+      </c>
+      <c r="AL6" s="4">
+        <v>37</v>
+      </c>
+      <c r="AM6" s="4">
+        <v>38</v>
+      </c>
+      <c r="AN6" s="4">
+        <v>39</v>
+      </c>
+      <c r="AO6" s="4">
+        <v>40</v>
+      </c>
+      <c r="AP6" s="4">
+        <v>41</v>
+      </c>
+      <c r="AQ6" s="4">
+        <v>42</v>
+      </c>
+      <c r="AR6" s="4">
+        <v>43</v>
+      </c>
+      <c r="AS6" s="4">
+        <v>44</v>
+      </c>
+      <c r="AT6" s="4">
+        <v>45</v>
+      </c>
+      <c r="AU6" s="4">
+        <v>46</v>
+      </c>
+      <c r="AV6" s="4">
+        <v>47</v>
+      </c>
+      <c r="AW6" s="4">
+        <v>48</v>
+      </c>
+      <c r="AX6" s="4">
+        <v>49</v>
+      </c>
+      <c r="AY6" s="4">
+        <v>50</v>
+      </c>
+      <c r="AZ6" s="4">
+        <v>51</v>
+      </c>
+      <c r="BA6" s="4">
+        <v>52</v>
+      </c>
+      <c r="BB6" s="4">
+        <v>53</v>
+      </c>
+      <c r="BC6" s="4">
+        <v>54</v>
+      </c>
+      <c r="BD6" s="4">
+        <v>55</v>
+      </c>
+      <c r="BE6" s="4">
+        <v>56</v>
+      </c>
+      <c r="BF6" s="4">
+        <v>57</v>
+      </c>
+      <c r="BG6" s="4">
+        <v>58</v>
+      </c>
+      <c r="BH6" s="4">
+        <v>59</v>
+      </c>
+      <c r="BI6" s="4">
+        <v>60</v>
+      </c>
+      <c r="BJ6" s="4">
+        <v>61</v>
+      </c>
+      <c r="BK6" s="4">
+        <v>62</v>
+      </c>
+      <c r="BL6" s="4">
+        <v>63</v>
+      </c>
+      <c r="BM6" s="4">
+        <v>64</v>
+      </c>
+      <c r="BN6" s="4">
+        <v>65</v>
+      </c>
+      <c r="BO6" s="4">
+        <v>66</v>
+      </c>
+      <c r="BP6" s="4">
+        <v>67</v>
+      </c>
+      <c r="BQ6" s="4">
+        <v>68</v>
+      </c>
+      <c r="BR6" s="4">
+        <v>69</v>
+      </c>
+      <c r="BS6" s="4">
+        <v>70</v>
+      </c>
+      <c r="BT6" s="4">
+        <v>71</v>
+      </c>
+      <c r="BU6" s="4">
+        <v>72</v>
+      </c>
+      <c r="BV6" s="4">
+        <v>73</v>
+      </c>
+      <c r="BW6" s="4">
+        <v>74</v>
+      </c>
+      <c r="BX6" s="4">
+        <v>75</v>
+      </c>
+      <c r="BY6" s="4">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1013,8 +1595,8 @@
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E3:AJ3"/>
-    <mergeCell ref="D2:AJ2"/>
+    <mergeCell ref="D2:BY2"/>
+    <mergeCell ref="E3:BY3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
 </worksheet>

</xml_diff>